<commit_message>
Update 092525 - Github Rule Code Locator.xlsx
</commit_message>
<xml_diff>
--- a/092525 - Github Rule Code Locator.xlsx
+++ b/092525 - Github Rule Code Locator.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JayAppell\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JayAppell\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32192011-DFB4-4543-A4B0-77BC16A9397E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{67EFDB37-0981-41E7-837E-44E1D2C1E68A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="62055" yWindow="1125" windowWidth="28800" windowHeight="20055" xr2:uid="{437B34C8-15BC-4035-9633-C13BCDFC4151}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="28800" windowHeight="15370" xr2:uid="{437B34C8-15BC-4035-9633-C13BCDFC4151}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -349,10 +348,10 @@
     <t>Github Providser</t>
   </si>
   <si>
-    <t>The Grey Alien Github Code Links (Click Link to view code)</t>
-  </si>
-  <si>
-    <t>Orendain's Github Code Links  (Click Link to view code)</t>
+    <t>The Grey Alien Github Code Links                      (Click Link to view code)</t>
+  </si>
+  <si>
+    <t>Orendain Github Code Links (Click Link to view code)</t>
   </si>
 </sst>
 </file>
@@ -416,13 +415,13 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -438,13 +437,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{902EFC5C-812F-4749-A8DD-268B4A13820C}" name="Table1" displayName="Table1" ref="A1:D103" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{902EFC5C-812F-4749-A8DD-268B4A13820C}" name="Table1" displayName="Table1" ref="A1:D103" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:D103" xr:uid="{902EFC5C-812F-4749-A8DD-268B4A13820C}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B35BA5D7-CCEC-45BE-AD8C-66F27B455D47}" name="Github Provider"/>
-    <tableColumn id="2" xr3:uid="{A2B1AF6D-2FC9-4363-9326-0045D34D7237}" name="Orendain's Github Code Links  (Click Link to view code)" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="2" xr3:uid="{A2B1AF6D-2FC9-4363-9326-0045D34D7237}" name="The Grey Alien Github Code Links                      (Click Link to view code)" dataDxfId="1" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{A65BBD55-7A97-448B-969F-2B428271F0CE}" name="Github Providser"/>
-    <tableColumn id="4" xr3:uid="{042613FE-E096-40EE-806E-5D8205BB6A0D}" name="The Grey Alien Github Code Links (Click Link to view code)" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="4" xr3:uid="{042613FE-E096-40EE-806E-5D8205BB6A0D}" name="Orendain Github Code Links (Click Link to view code)" dataDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -762,13 +761,13 @@
         <v>105</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>106</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>